<commit_message>
cuartocomit creacion xls y docx
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,11 +431,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>guitarra</t>
+          <t>azul</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>marron</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
quinto comit creacion xls, docx y pdf
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,31 +431,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>azul</t>
+          <t>camara</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rojo</t>
+          <t>dvr</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>marron</t>
+          <t>bobinas de cable</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sexto comit creacion xls, docx, pdf y cmbinacion de archvos
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -451,7 +451,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bobinas de cable</t>
+          <t>bobina de cable</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -461,7 +461,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>swith</t>
         </is>
       </c>
       <c r="B5" t="n">

</xml_diff>